<commit_message>
feat: Config_Types covers all datatypes; add TOML golden + parser fixes (#84)
- expand Config_Types.xlsx: adds DataType=credential/asset rows, typed
  OrchestratorAsset sheet, and a _TargetType sheet (Targets → ToTargetConfig)
- add Config_Types.toml fixture covering string, int, double, bool,
  DateOnly, DateTime, TimeOnly, typed assets, and _TargetType
- fix parseTomlNode: smol-toml local-date/time objects were matched by
  the generic "recurse as child" branch; add explicit temporal-object
  check before the object branch so dates become scalar properties
- fix parseTomlNode: pass valueType from TOML asset objects so typed
  assets (valueType=string/int/bool) generate correctly typed properties
- add Config_Types.toml entry to run-generators.mjs (stem Config_Types_Toml)
- update goldens: Config_Types.cs/.xaml (expanded), Config_Types_Toml.cs/.xaml (new)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test/fixtures/Config_Types.xlsx
+++ b/test/fixtures/Config_Types.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Settings" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Constants" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Assets" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Targets" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,6 +445,11 @@
           <t>Description</t>
         </is>
       </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>DataType</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -549,6 +555,50 @@
       <c r="C8" t="inlineStr">
         <is>
           <t>TimeOnly — time only, no date</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>SapCredential</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Default/cred_sap_types</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>SAP Orchestrator credential.</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>credential</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>QueueNameRef</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Default/cfgtree_queue_types</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Queue name Orchestrator asset.</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>asset</t>
         </is>
       </c>
     </row>
@@ -699,7 +749,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -723,6 +773,11 @@
           <t>Description</t>
         </is>
       </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>ValueType</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -765,6 +820,177 @@
       <c r="D3" t="inlineStr">
         <is>
           <t>FTP server credential.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>QueueNameAsset</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>cfgtree_queue_name_types</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>ConFigTree/Test</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Input queue name.</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>MaxItemsAsset</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>cfgtree_max_items_types</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ConFigTree/Test</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Max items to process.</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>StrictModeAsset</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>cfgtree_strict_mode_types</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>ConFigTree/Test</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Strict processing toggle.</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>_TargetType</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Acme.External.TargetConfig</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Host</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>targets.example.com</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Target host address.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Port</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>8080</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Target port number.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Enabled</t>
+        </is>
+      </c>
+      <c r="B5" t="b">
+        <v>1</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Enable target connection.</t>
         </is>
       </c>
     </row>

</xml_diff>